<commit_message>
ui code refactor in progress
</commit_message>
<xml_diff>
--- a/docs/weapon_active_skill_design.xlsx
+++ b/docs/weapon_active_skill_design.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主动技能设计" sheetId="1" r:id="Rbd1b781242c24074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主动技能设计" sheetId="1" r:id="Rb50f884cc12e443d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -498,7 +498,7 @@
     </x:row>
     <x:row r="3" ht="31" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>说明：解锁条件与专属主动技能均为拟定设计，尚未实装；解锁条件采用“武器 Lv.3 + 本局首次完成核心被动循环”的统一原则。</x:v>
+        <x:v>说明：解锁条件与专属主动技能均为拟定设计，尚未实装。统一规则为“武器 Lv.3 + 本局已触发过 1 次该武器特长”，两个条件独立记录、顺序不限。条件栏第一行用于界面显示，第二行说明详细触发判定。</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -537,7 +537,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D6" s="30" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次积满 10 层长矛充能并开始换弹后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 长矛充能 0/1
+详细判定：长矛充能首次积满 10 层，并进入换弹。</x:v>
       </x:c>
       <x:c r="E6" s="42" t="str">
         <x:v>Blade Recall / 万刃归流</x:v>
@@ -557,7 +558,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D7" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次完成 5 秒副手蓄力后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 副手蓄力 0/1
+详细判定：副手连续蓄力达到 5 秒，并完成蓄力。</x:v>
       </x:c>
       <x:c r="E7" s="43" t="str">
         <x:v>Siege Breach / 攻城破口</x:v>
@@ -577,7 +579,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D8" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次达成 10 次连续命中后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 连续命中 0/1
+详细判定：链锯发射器连续命中达到 10 次。</x:v>
       </x:c>
       <x:c r="E8" s="43" t="str">
         <x:v>Predator Chain / 猎杀链锯</x:v>
@@ -597,7 +600,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D9" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次完成一次满武器能量释放后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 满能量释放 0/1
+详细判定：武器能量充满后，完成 1 次能量释放。</x:v>
       </x:c>
       <x:c r="E9" s="43" t="str">
         <x:v>Resonance Lance / 共振长束</x:v>
@@ -617,7 +621,8 @@
         <x:v>被动已实装；不可选为主武器；当前仍可通过槽位长按请求通用主动技能</x:v>
       </x:c>
       <x:c r="D10" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次达成 6 次连续冲刺刃命中后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 连续冲刺斩击 0/1
+详细判定：冲刺刃连续命中达到 6 次。</x:v>
       </x:c>
       <x:c r="E10" s="43" t="str">
         <x:v>Return Execution / 往返处决</x:v>
@@ -637,7 +642,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D11" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次消耗完整四个弹匣阶段后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 完整热量循环 0/1
+详细判定：连续消耗完四个弹匣阶段。</x:v>
       </x:c>
       <x:c r="E11" s="43" t="str">
         <x:v>Thermal Overflow / 热流溢出</x:v>
@@ -657,7 +663,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D12" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次消费 Cold Snap 后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 寒潮 0/1
+详细判定：积累并消费 1 次 Cold Snap。</x:v>
       </x:c>
       <x:c r="E12" s="43" t="str">
         <x:v>Whiteout Field / 白障领域</x:v>
@@ -677,7 +684,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D13" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次完成一次满能量 Focus Channel 后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 聚焦通道 0/1
+详细判定：武器能量充满后，完成 1 次 Focus Channel。</x:v>
       </x:c>
       <x:c r="E13" s="43" t="str">
         <x:v>Perfect Focus / 完美聚焦</x:v>
@@ -697,7 +705,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D14" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次以 4 层充能开始换弹后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 满层换弹 0/1
+详细判定：持有 4 层充能时开始换弹。</x:v>
       </x:c>
       <x:c r="E14" s="43" t="str">
         <x:v>Belt-Fed Suppression / 弹链压制</x:v>
@@ -717,7 +726,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D15" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次完成武器入场强化部署后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 强化部署 0/1
+详细判定：武器入场后完成 1 次强化卫星部署。</x:v>
       </x:c>
       <x:c r="E15" s="43" t="str">
         <x:v>Orbital Recall / 轨道召回</x:v>
@@ -737,7 +747,8 @@
         <x:v>被动已实装；不可选为主武器；当前仍可通过槽位长按请求通用主动技能</x:v>
       </x:c>
       <x:c r="D16" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次达成 6 次连续命中并开启标记窗口后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 连续命中标记 0/1
+详细判定：连续命中达到 6 次，并开启标记窗口。</x:v>
       </x:c>
       <x:c r="E16" s="43" t="str">
         <x:v>Arc Designation / 电弧标定</x:v>
@@ -757,7 +768,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D17" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次完成满能量 Plasma Discharge 后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 等离子释放 0/1
+详细判定：武器能量充满后，完成 1 次 Plasma Discharge。</x:v>
       </x:c>
       <x:c r="E17" s="43" t="str">
         <x:v>Rift Impalement / 裂隙贯穿</x:v>
@@ -777,7 +789,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D18" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次由该武器完成 3 次击杀后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 连续击杀 0/1
+详细判定：由火箭发射器累计完成 3 次击杀。</x:v>
       </x:c>
       <x:c r="E18" s="43" t="str">
         <x:v>Cluster Barrage / 集束弹幕</x:v>
@@ -797,7 +810,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D19" s="31" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次完成一次 Crossfire 破防后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 交叉火力破防 0/1
+详细判定：触发 1 次 Crossfire，并由其完成破防。</x:v>
       </x:c>
       <x:c r="E19" s="43" t="str">
         <x:v>Breach Volley / 突破齐射</x:v>
@@ -817,7 +831,8 @@
         <x:v>被动已实装；当前使用通用主动技能占位</x:v>
       </x:c>
       <x:c r="D20" s="32" t="str">
-        <x:v>拟定：武器达到 Lv.3，且本局首次消费 5 秒副手蓄力或 Crossfire 蓄势后解锁</x:v>
+        <x:v>界面显示：武器 Lv.3 + 满蓄势射击 0/1
+详细判定：消费 5 秒副手蓄力或完整 Crossfire 蓄势，完成 1 次射击。</x:v>
       </x:c>
       <x:c r="E20" s="44" t="str">
         <x:v>Deadeye Protocol / 死眼协议</x:v>
@@ -834,7 +849,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa00404ddbc452f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c68097179334a33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>